<commit_message>
8. Google Services Connect, EventManager Add
이벤트 매니저 추가, BaseEvent를 통해 Choice에서 Event를 실행할 수 있도록 함.
추가적인 이벤트를 개발하여 다양성을 늘릴 수 있을 것으로 기대.
추가적으로 Google Service와 연동.
keyStore는 kguwarlike
</commit_message>
<xml_diff>
--- a/Assets/Resources/NodeData.xlsx
+++ b/Assets/Resources/NodeData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\monke\Desktop\war_LIke2\Assets\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE53D865-782C-4A2B-A971-D30840B02CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FAE9BA8-5A09-4FBC-B46D-2EA1FD22DC9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28690" yWindow="5890" windowWidth="19420" windowHeight="11500" xr2:uid="{D00B35EE-5D9B-470B-AFB3-7D5F75EB546F}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{D00B35EE-5D9B-470B-AFB3-7D5F75EB546F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="49">
   <si>
     <t>1장</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -79,10 +79,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>EventSuccessRate</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>EventStack</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -220,6 +216,10 @@
   </si>
   <si>
     <t>테스터의 승리</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BaseEvent</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -707,6 +707,30 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -714,30 +738,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1064,51 +1064,51 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
-      <c r="J1" s="45"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="45"/>
-      <c r="M1" s="45"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
     </row>
     <row r="2" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A2" s="10" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="46" t="s">
+      <c r="D2" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
-      <c r="H2" s="46"/>
-      <c r="I2" s="46"/>
-      <c r="J2" s="46"/>
-      <c r="K2" s="46"/>
-      <c r="L2" s="46"/>
-      <c r="M2" s="46"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
     </row>
     <row r="3" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="41"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="38"/>
       <c r="D3" s="28" t="s">
         <v>7</v>
       </c>
@@ -1119,13 +1119,13 @@
         <v>9</v>
       </c>
       <c r="G3" s="15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H3" s="15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J3" s="15"/>
       <c r="K3" s="15"/>
@@ -1175,28 +1175,28 @@
       <c r="BC3" s="2"/>
     </row>
     <row r="4" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="41"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
       <c r="D4" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>39</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
@@ -1246,28 +1246,28 @@
       <c r="BC4" s="2"/>
     </row>
     <row r="5" spans="1:55" s="18" customFormat="1" ht="68.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="38"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="46"/>
       <c r="D5" s="16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I5" s="17" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J5" s="17"/>
       <c r="K5" s="17"/>
@@ -1317,11 +1317,11 @@
       <c r="BC5" s="17"/>
     </row>
     <row r="6" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A6" s="39" t="s">
+      <c r="A6" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="41"/>
+      <c r="B6" s="37"/>
+      <c r="C6" s="38"/>
       <c r="D6" s="3">
         <v>0</v>
       </c>
@@ -1388,28 +1388,28 @@
       <c r="BC6" s="2"/>
     </row>
     <row r="7" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="40"/>
-      <c r="C7" s="41"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="38"/>
       <c r="D7" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
@@ -1460,10 +1460,10 @@
     </row>
     <row r="8" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A8" s="22"/>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="43"/>
+      <c r="C8" s="40"/>
       <c r="D8" s="3"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -1524,10 +1524,10 @@
       </c>
       <c r="C9" s="30"/>
       <c r="D9" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1702,7 +1702,7 @@
       <c r="A12" s="23"/>
       <c r="B12" s="12"/>
       <c r="C12" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="2"/>
@@ -1768,7 +1768,7 @@
       <c r="D13" s="16"/>
       <c r="E13" s="17"/>
       <c r="F13" s="17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G13" s="17"/>
       <c r="H13" s="17"/>
@@ -1829,7 +1829,7 @@
       <c r="D14" s="3"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -1885,7 +1885,7 @@
       <c r="A15" s="23"/>
       <c r="B15" s="13"/>
       <c r="C15" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D15" s="3"/>
       <c r="E15" s="2"/>
@@ -1944,7 +1944,7 @@
       <c r="A16" s="23"/>
       <c r="B16" s="13"/>
       <c r="C16" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D16" s="3"/>
       <c r="E16" s="2"/>
@@ -2003,7 +2003,7 @@
       <c r="A17" s="23"/>
       <c r="B17" s="13"/>
       <c r="C17" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D17" s="3"/>
       <c r="E17" s="2"/>
@@ -2062,7 +2062,7 @@
       <c r="A18" s="23"/>
       <c r="B18" s="13"/>
       <c r="C18" s="9" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="2"/>
@@ -2126,7 +2126,7 @@
       <c r="D19" s="16"/>
       <c r="E19" s="17"/>
       <c r="F19" s="17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G19" s="17"/>
       <c r="H19" s="17"/>
@@ -2187,7 +2187,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -2243,7 +2243,7 @@
       <c r="A21" s="23"/>
       <c r="B21" s="13"/>
       <c r="C21" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D21" s="3"/>
       <c r="E21" s="2"/>
@@ -2302,7 +2302,7 @@
       <c r="A22" s="23"/>
       <c r="B22" s="13"/>
       <c r="C22" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D22" s="3"/>
       <c r="E22" s="2"/>
@@ -2361,7 +2361,7 @@
       <c r="A23" s="23"/>
       <c r="B23" s="13"/>
       <c r="C23" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D23" s="3"/>
       <c r="E23" s="2"/>
@@ -2420,7 +2420,7 @@
       <c r="A24" s="23"/>
       <c r="B24" s="13"/>
       <c r="C24" s="9" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="2"/>
@@ -2484,7 +2484,7 @@
       <c r="D25" s="16"/>
       <c r="E25" s="17"/>
       <c r="F25" s="17" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G25" s="17"/>
       <c r="H25" s="17"/>
@@ -2545,7 +2545,7 @@
       <c r="D26" s="3"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -2601,7 +2601,7 @@
       <c r="A27" s="23"/>
       <c r="B27" s="13"/>
       <c r="C27" s="8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D27" s="3"/>
       <c r="E27" s="2"/>
@@ -2660,7 +2660,7 @@
       <c r="A28" s="23"/>
       <c r="B28" s="13"/>
       <c r="C28" s="8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="2"/>
@@ -2719,7 +2719,7 @@
       <c r="A29" s="23"/>
       <c r="B29" s="13"/>
       <c r="C29" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29" s="3"/>
       <c r="E29" s="2"/>
@@ -2778,7 +2778,7 @@
       <c r="A30" s="23"/>
       <c r="B30" s="14"/>
       <c r="C30" s="9" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="D30" s="3"/>
       <c r="E30" s="2"/>
@@ -2836,7 +2836,7 @@
     <row r="31" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A31" s="23"/>
       <c r="B31" s="31" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C31" s="32"/>
       <c r="D31" s="3"/>
@@ -2895,14 +2895,14 @@
     <row r="32" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A32" s="23"/>
       <c r="B32" s="35" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C32" s="35"/>
       <c r="D32" s="3"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
@@ -2956,14 +2956,14 @@
     <row r="33" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A33" s="23"/>
       <c r="B33" s="35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C33" s="35"/>
       <c r="D33" s="3"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
@@ -3017,14 +3017,14 @@
     <row r="34" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A34" s="23"/>
       <c r="B34" s="35" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C34" s="35"/>
       <c r="D34" s="3"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
@@ -3078,7 +3078,7 @@
     <row r="35" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A35" s="25"/>
       <c r="B35" s="31" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C35" s="32"/>
       <c r="D35" s="3"/>
@@ -3137,7 +3137,7 @@
     <row r="36" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A36" s="26"/>
       <c r="B36" s="29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C36" s="30"/>
       <c r="D36" s="3"/>
@@ -3145,7 +3145,7 @@
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
@@ -3257,7 +3257,7 @@
     <row r="38" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A38" s="26"/>
       <c r="C38" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="2"/>
@@ -3324,7 +3324,7 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
       <c r="H39" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I39" s="17"/>
       <c r="J39" s="17"/>
@@ -3384,7 +3384,7 @@
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
@@ -3437,7 +3437,7 @@
     <row r="41" spans="1:55" x14ac:dyDescent="0.6">
       <c r="A41" s="26"/>
       <c r="C41" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D41" s="3"/>
       <c r="E41" s="2"/>
@@ -3495,7 +3495,7 @@
     <row r="42" spans="1:55" x14ac:dyDescent="0.6">
       <c r="A42" s="26"/>
       <c r="C42" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D42" s="3"/>
       <c r="E42" s="2"/>
@@ -3553,7 +3553,7 @@
     <row r="43" spans="1:55" x14ac:dyDescent="0.6">
       <c r="A43" s="26"/>
       <c r="C43" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D43" s="3"/>
       <c r="E43" s="2"/>
@@ -3611,15 +3611,13 @@
     <row r="44" spans="1:55" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A44" s="26"/>
       <c r="C44" s="5" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
-      <c r="H44" s="2">
-        <v>0.5</v>
-      </c>
+      <c r="H44" s="2"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
@@ -3678,7 +3676,7 @@
       <c r="F45" s="17"/>
       <c r="G45" s="17"/>
       <c r="H45" s="17" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I45" s="17"/>
       <c r="J45" s="17"/>
@@ -3737,7 +3735,9 @@
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
+      <c r="H46" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
@@ -3789,7 +3789,7 @@
     <row r="47" spans="1:55" x14ac:dyDescent="0.6">
       <c r="A47" s="26"/>
       <c r="C47" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D47" s="3"/>
       <c r="E47" s="2"/>
@@ -3847,7 +3847,7 @@
     <row r="48" spans="1:55" x14ac:dyDescent="0.6">
       <c r="A48" s="26"/>
       <c r="C48" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D48" s="3"/>
       <c r="E48" s="2"/>
@@ -3905,7 +3905,7 @@
     <row r="49" spans="1:55" x14ac:dyDescent="0.6">
       <c r="A49" s="26"/>
       <c r="C49" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D49" s="3"/>
       <c r="E49" s="2"/>
@@ -3963,15 +3963,13 @@
     <row r="50" spans="1:55" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A50" s="26"/>
       <c r="C50" s="5" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="D50" s="3"/>
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
-      <c r="H50" s="2">
-        <v>0.5</v>
-      </c>
+      <c r="H50" s="2"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
@@ -4030,7 +4028,7 @@
       <c r="F51" s="17"/>
       <c r="G51" s="17"/>
       <c r="H51" s="17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I51" s="17"/>
       <c r="J51" s="17"/>
@@ -4089,7 +4087,9 @@
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
-      <c r="H52" s="2"/>
+      <c r="H52" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
@@ -4141,7 +4141,7 @@
     <row r="53" spans="1:55" x14ac:dyDescent="0.6">
       <c r="A53" s="26"/>
       <c r="C53" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D53" s="3"/>
       <c r="E53" s="2"/>
@@ -4199,7 +4199,7 @@
     <row r="54" spans="1:55" x14ac:dyDescent="0.6">
       <c r="A54" s="26"/>
       <c r="C54" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D54" s="3"/>
       <c r="E54" s="2"/>
@@ -4257,7 +4257,7 @@
     <row r="55" spans="1:55" x14ac:dyDescent="0.6">
       <c r="A55" s="26"/>
       <c r="C55" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D55" s="3"/>
       <c r="E55" s="2"/>
@@ -4315,15 +4315,13 @@
     <row r="56" spans="1:55" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A56" s="26"/>
       <c r="C56" s="11" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
-      <c r="H56" s="2">
-        <v>0.5</v>
-      </c>
+      <c r="H56" s="2"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
@@ -4375,7 +4373,7 @@
     <row r="57" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A57" s="26"/>
       <c r="B57" s="31" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C57" s="32"/>
       <c r="D57" s="3"/>
@@ -4434,7 +4432,7 @@
     <row r="58" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A58" s="26"/>
       <c r="B58" s="29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C58" s="30"/>
       <c r="D58" s="3"/>
@@ -4443,7 +4441,7 @@
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>

</xml_diff>

<commit_message>
9. Base Devlopment Finish
</commit_message>
<xml_diff>
--- a/Assets/Resources/NodeData.xlsx
+++ b/Assets/Resources/NodeData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\monke\Desktop\war_LIke2\Assets\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FAE9BA8-5A09-4FBC-B46D-2EA1FD22DC9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BB12DA6-5BFC-4156-A963-D63BF5CB2396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{D00B35EE-5D9B-470B-AFB3-7D5F75EB546F}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="52">
   <si>
     <t>1장</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -220,6 +220,18 @@
   </si>
   <si>
     <t>BaseEvent</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>StrUp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DexUp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ConUp</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -685,18 +697,51 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -705,39 +750,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1064,21 +1076,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="42"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
     </row>
     <row r="2" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A2" s="10" t="s">
@@ -1090,25 +1102,25 @@
       <c r="C2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="43" t="s">
+      <c r="D2" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="43"/>
-      <c r="F2" s="43"/>
-      <c r="G2" s="43"/>
-      <c r="H2" s="43"/>
-      <c r="I2" s="43"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
-      <c r="L2" s="43"/>
-      <c r="M2" s="43"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+      <c r="K2" s="31"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
     </row>
     <row r="3" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="37"/>
-      <c r="C3" s="38"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="34"/>
       <c r="D3" s="28" t="s">
         <v>7</v>
       </c>
@@ -1175,11 +1187,11 @@
       <c r="BC3" s="2"/>
     </row>
     <row r="4" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="37"/>
-      <c r="C4" s="38"/>
+      <c r="B4" s="33"/>
+      <c r="C4" s="34"/>
       <c r="D4" s="3" t="s">
         <v>26</v>
       </c>
@@ -1246,11 +1258,11 @@
       <c r="BC4" s="2"/>
     </row>
     <row r="5" spans="1:55" s="18" customFormat="1" ht="68.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="46"/>
+      <c r="B5" s="36"/>
+      <c r="C5" s="37"/>
       <c r="D5" s="16" t="s">
         <v>27</v>
       </c>
@@ -1317,11 +1329,11 @@
       <c r="BC5" s="17"/>
     </row>
     <row r="6" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="37"/>
-      <c r="C6" s="38"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="34"/>
       <c r="D6" s="3">
         <v>0</v>
       </c>
@@ -1388,11 +1400,11 @@
       <c r="BC6" s="2"/>
     </row>
     <row r="7" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A7" s="36" t="s">
+      <c r="A7" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="37"/>
-      <c r="C7" s="38"/>
+      <c r="B7" s="33"/>
+      <c r="C7" s="34"/>
       <c r="D7" s="3" t="s">
         <v>28</v>
       </c>
@@ -1460,10 +1472,10 @@
     </row>
     <row r="8" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A8" s="22"/>
-      <c r="B8" s="39" t="s">
+      <c r="B8" s="40" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="40"/>
+      <c r="C8" s="41"/>
       <c r="D8" s="3"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -1519,10 +1531,10 @@
     </row>
     <row r="9" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A9" s="23"/>
-      <c r="B9" s="29" t="s">
+      <c r="B9" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="30"/>
+      <c r="C9" s="43"/>
       <c r="D9" s="3" t="s">
         <v>29</v>
       </c>
@@ -1582,10 +1594,10 @@
     </row>
     <row r="10" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A10" s="23"/>
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="32"/>
+      <c r="C10" s="39"/>
       <c r="D10" s="3"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -1641,10 +1653,10 @@
     </row>
     <row r="11" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A11" s="23"/>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="44" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="34"/>
+      <c r="C11" s="45"/>
       <c r="D11" s="3"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -2835,10 +2847,10 @@
     </row>
     <row r="31" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A31" s="23"/>
-      <c r="B31" s="31" t="s">
+      <c r="B31" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="C31" s="32"/>
+      <c r="C31" s="39"/>
       <c r="D31" s="3"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
@@ -2894,10 +2906,10 @@
     </row>
     <row r="32" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A32" s="23"/>
-      <c r="B32" s="35" t="s">
+      <c r="B32" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="35"/>
+      <c r="C32" s="46"/>
       <c r="D32" s="3"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
@@ -2955,10 +2967,10 @@
     </row>
     <row r="33" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A33" s="23"/>
-      <c r="B33" s="35" t="s">
+      <c r="B33" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="35"/>
+      <c r="C33" s="46"/>
       <c r="D33" s="3"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
@@ -3016,10 +3028,10 @@
     </row>
     <row r="34" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A34" s="23"/>
-      <c r="B34" s="35" t="s">
+      <c r="B34" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="35"/>
+      <c r="C34" s="46"/>
       <c r="D34" s="3"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
@@ -3077,10 +3089,10 @@
     </row>
     <row r="35" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A35" s="25"/>
-      <c r="B35" s="31" t="s">
+      <c r="B35" s="38" t="s">
         <v>22</v>
       </c>
-      <c r="C35" s="32"/>
+      <c r="C35" s="39"/>
       <c r="D35" s="3"/>
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
@@ -3136,10 +3148,10 @@
     </row>
     <row r="36" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A36" s="26"/>
-      <c r="B36" s="29" t="s">
+      <c r="B36" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="C36" s="30"/>
+      <c r="C36" s="43"/>
       <c r="D36" s="3"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
@@ -3197,10 +3209,10 @@
     </row>
     <row r="37" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A37" s="26"/>
-      <c r="B37" s="29" t="s">
+      <c r="B37" s="42" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="30"/>
+      <c r="C37" s="43"/>
       <c r="D37" s="3"/>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
@@ -3501,7 +3513,9 @@
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
-      <c r="H42" s="2"/>
+      <c r="H42" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
@@ -3853,7 +3867,9 @@
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
-      <c r="H48" s="2"/>
+      <c r="H48" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
@@ -4205,7 +4221,9 @@
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
-      <c r="H54" s="2"/>
+      <c r="H54" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
@@ -4372,10 +4390,10 @@
     </row>
     <row r="57" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A57" s="26"/>
-      <c r="B57" s="31" t="s">
+      <c r="B57" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="C57" s="32"/>
+      <c r="C57" s="39"/>
       <c r="D57" s="3"/>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
@@ -4431,10 +4449,10 @@
     </row>
     <row r="58" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A58" s="26"/>
-      <c r="B58" s="29" t="s">
+      <c r="B58" s="42" t="s">
         <v>25</v>
       </c>
-      <c r="C58" s="30"/>
+      <c r="C58" s="43"/>
       <c r="D58" s="3"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
@@ -4493,16 +4511,6 @@
     <row r="59" spans="1:55" ht="17.25" thickTop="1" x14ac:dyDescent="0.6"/>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="D2:M2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B57:C57"/>
@@ -4513,6 +4521,16 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="D2:M2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
10. Meeting Event Add, Event structure Fixed
조우 이벤트 생성, nodeData, statusData 수정.
Event 구조 변경. BaseEvent에서 추상 클래스 2개 선언. 다형성 구현 완료. Execute()에서 nextNode를 입력 여부에 따라 실행 내용 변동 가능.
</commit_message>
<xml_diff>
--- a/Assets/Resources/NodeData.xlsx
+++ b/Assets/Resources/NodeData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\monke\Desktop\war_LIke2\Assets\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BB12DA6-5BFC-4156-A963-D63BF5CB2396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929A5889-BB97-4F5F-9ACC-D7F0DF0C7ED2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{D00B35EE-5D9B-470B-AFB3-7D5F75EB546F}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="74">
   <si>
     <t>1장</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -119,10 +119,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>EventName</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>EndingNode</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -167,10 +163,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>엔딩 노드 확인하러 가기.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Combat_01</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -187,18 +179,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>E_001</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>이벤트 노드에 진입하였다. 당신의 운을 확인한다. 각 이벤트 발생 확률은 50%이다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>스탯 상승 이벤트</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>힘이 상승한다.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -232,6 +216,110 @@
   </si>
   <si>
     <t>ConUp</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EventCategory</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>스탯 상승</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ending_02</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>테스터의 패배</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>당신은 사망하였다. 당신의 나약함은 멸망한 세상에서 도태되기 충분하였고 당신은 노숙자와의 전투 끝에 생을 마감하였다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EventNode</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Event_02</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조우 이벤트 발생. \n 당신은 굶주린 모녀와 마주하였다. 어떻게 할 것인가?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>서울</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>조우</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>무시한다. (아무런 일도 일어나지 않음.)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Main_03</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>두번째 이벤드 노드 확인하러 가기</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Event_02</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>무시하기_굶주린모녀</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전투하기_굶주린모녀</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>도와주기_굶주린모녀</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CombatNode</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Combat_02</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>전투에 돌입한다. 당신의 상대는 굶주린 모녀이다. 해치워라.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ending_01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_003</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>E_000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>싸운다. (돈 +10000원 통조림 + 1)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>도와준다. (통조림 - 2 선행 + 1)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -697,6 +785,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -707,15 +831,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -723,33 +838,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1076,21 +1164,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30"/>
-      <c r="H1" s="30"/>
-      <c r="I1" s="30"/>
-      <c r="J1" s="30"/>
-      <c r="K1" s="30"/>
-      <c r="L1" s="30"/>
-      <c r="M1" s="30"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
     </row>
     <row r="2" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A2" s="10" t="s">
@@ -1102,25 +1190,25 @@
       <c r="C2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="31" t="s">
+      <c r="D2" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
-      <c r="K2" s="31"/>
-      <c r="L2" s="31"/>
-      <c r="M2" s="31"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
+      <c r="H2" s="43"/>
+      <c r="I2" s="43"/>
+      <c r="J2" s="43"/>
+      <c r="K2" s="43"/>
+      <c r="L2" s="43"/>
+      <c r="M2" s="43"/>
     </row>
     <row r="3" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A3" s="32" t="s">
+      <c r="A3" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="33"/>
-      <c r="C3" s="34"/>
+      <c r="B3" s="37"/>
+      <c r="C3" s="38"/>
       <c r="D3" s="28" t="s">
         <v>7</v>
       </c>
@@ -1137,11 +1225,17 @@
         <v>22</v>
       </c>
       <c r="I3" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
+        <v>23</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>66</v>
+      </c>
       <c r="M3" s="15"/>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -1187,32 +1281,38 @@
       <c r="BC3" s="2"/>
     </row>
     <row r="4" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="34"/>
+      <c r="B4" s="37"/>
+      <c r="C4" s="38"/>
       <c r="D4" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
+      <c r="J4" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="M4" s="2"/>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -1257,33 +1357,39 @@
       <c r="BB4" s="2"/>
       <c r="BC4" s="2"/>
     </row>
-    <row r="5" spans="1:55" s="18" customFormat="1" ht="68.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A5" s="35" t="s">
+    <row r="5" spans="1:55" s="18" customFormat="1" ht="102" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A5" s="44" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="36"/>
-      <c r="C5" s="37"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="46"/>
       <c r="D5" s="16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="I5" s="17" t="s">
-        <v>46</v>
-      </c>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
+        <v>42</v>
+      </c>
+      <c r="J5" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="L5" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="M5" s="17"/>
       <c r="N5" s="17"/>
       <c r="O5" s="17"/>
@@ -1329,11 +1435,11 @@
       <c r="BC5" s="17"/>
     </row>
     <row r="6" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="33"/>
-      <c r="C6" s="34"/>
+      <c r="B6" s="37"/>
+      <c r="C6" s="38"/>
       <c r="D6" s="3">
         <v>0</v>
       </c>
@@ -1352,9 +1458,15 @@
       <c r="I6" s="2">
         <v>72</v>
       </c>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
+      <c r="J6" s="2">
+        <v>72</v>
+      </c>
+      <c r="K6" s="2">
+        <v>2</v>
+      </c>
+      <c r="L6" s="2">
+        <v>2</v>
+      </c>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -1400,32 +1512,38 @@
       <c r="BC6" s="2"/>
     </row>
     <row r="7" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A7" s="32" t="s">
+      <c r="A7" s="36" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="33"/>
-      <c r="C7" s="34"/>
+      <c r="B7" s="37"/>
+      <c r="C7" s="38"/>
       <c r="D7" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
+        <v>27</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="M7" s="2"/>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1472,10 +1590,10 @@
     </row>
     <row r="8" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A8" s="22"/>
-      <c r="B8" s="40" t="s">
+      <c r="B8" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="41"/>
+      <c r="C8" s="40"/>
       <c r="D8" s="3"/>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -1531,15 +1649,15 @@
     </row>
     <row r="9" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A9" s="23"/>
-      <c r="B9" s="42" t="s">
+      <c r="B9" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="43"/>
+      <c r="C9" s="30"/>
       <c r="D9" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1594,10 +1712,10 @@
     </row>
     <row r="10" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A10" s="23"/>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="39"/>
+      <c r="C10" s="32"/>
       <c r="D10" s="3"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -1653,10 +1771,10 @@
     </row>
     <row r="11" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A11" s="23"/>
-      <c r="B11" s="44" t="s">
+      <c r="B11" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="45"/>
+      <c r="C11" s="34"/>
       <c r="D11" s="3"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -1780,7 +1898,7 @@
       <c r="D13" s="16"/>
       <c r="E13" s="17"/>
       <c r="F13" s="17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G13" s="17"/>
       <c r="H13" s="17"/>
@@ -1841,7 +1959,7 @@
       <c r="D14" s="3"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -2074,7 +2192,7 @@
       <c r="A18" s="23"/>
       <c r="B18" s="13"/>
       <c r="C18" s="9" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D18" s="3"/>
       <c r="E18" s="2"/>
@@ -2138,7 +2256,7 @@
       <c r="D19" s="16"/>
       <c r="E19" s="17"/>
       <c r="F19" s="17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G19" s="17"/>
       <c r="H19" s="17"/>
@@ -2199,7 +2317,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -2432,7 +2550,7 @@
       <c r="A24" s="23"/>
       <c r="B24" s="13"/>
       <c r="C24" s="9" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="2"/>
@@ -2496,7 +2614,7 @@
       <c r="D25" s="16"/>
       <c r="E25" s="17"/>
       <c r="F25" s="17" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="G25" s="17"/>
       <c r="H25" s="17"/>
@@ -2557,7 +2675,7 @@
       <c r="D26" s="3"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2" t="s">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -2790,7 +2908,7 @@
       <c r="A30" s="23"/>
       <c r="B30" s="14"/>
       <c r="C30" s="9" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D30" s="3"/>
       <c r="E30" s="2"/>
@@ -2847,10 +2965,10 @@
     </row>
     <row r="31" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A31" s="23"/>
-      <c r="B31" s="38" t="s">
+      <c r="B31" s="31" t="s">
         <v>18</v>
       </c>
-      <c r="C31" s="39"/>
+      <c r="C31" s="32"/>
       <c r="D31" s="3"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
@@ -2906,21 +3024,23 @@
     </row>
     <row r="32" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A32" s="23"/>
-      <c r="B32" s="46" t="s">
+      <c r="B32" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="C32" s="46"/>
+      <c r="C32" s="35"/>
       <c r="D32" s="3"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="H32" s="2"/>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
       <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
+      <c r="L32" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -2967,21 +3087,23 @@
     </row>
     <row r="33" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A33" s="23"/>
-      <c r="B33" s="46" t="s">
+      <c r="B33" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="46"/>
+      <c r="C33" s="35"/>
       <c r="D33" s="3"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
+      <c r="L33" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="M33" s="2"/>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -3028,21 +3150,23 @@
     </row>
     <row r="34" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A34" s="23"/>
-      <c r="B34" s="46" t="s">
+      <c r="B34" s="35" t="s">
         <v>21</v>
       </c>
-      <c r="C34" s="46"/>
+      <c r="C34" s="35"/>
       <c r="D34" s="3"/>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2" t="s">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
+      <c r="L34" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="M34" s="2"/>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -3089,10 +3213,10 @@
     </row>
     <row r="35" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A35" s="25"/>
-      <c r="B35" s="38" t="s">
+      <c r="B35" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="C35" s="39"/>
+      <c r="C35" s="32"/>
       <c r="D35" s="3"/>
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
@@ -3148,20 +3272,22 @@
     </row>
     <row r="36" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A36" s="26"/>
-      <c r="B36" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="C36" s="43"/>
+      <c r="B36" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="C36" s="30"/>
       <c r="D36" s="3"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
+      <c r="K36" s="2" t="s">
+        <v>58</v>
+      </c>
       <c r="L36" s="2"/>
       <c r="M36" s="2"/>
       <c r="N36" s="2"/>
@@ -3209,10 +3335,10 @@
     </row>
     <row r="37" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A37" s="26"/>
-      <c r="B37" s="42" t="s">
+      <c r="B37" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="43"/>
+      <c r="C37" s="30"/>
       <c r="D37" s="3"/>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
@@ -3280,7 +3406,9 @@
       </c>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
+      <c r="K38" s="2">
+        <v>3</v>
+      </c>
       <c r="L38" s="2"/>
       <c r="M38" s="2"/>
       <c r="N38" s="2"/>
@@ -3326,7 +3454,7 @@
       <c r="BB38" s="2"/>
       <c r="BC38" s="2"/>
     </row>
-    <row r="39" spans="1:55" s="18" customFormat="1" ht="17.25" thickTop="1" x14ac:dyDescent="0.6">
+    <row r="39" spans="1:55" s="18" customFormat="1" ht="34.15" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A39" s="27"/>
       <c r="C39" s="21" t="s">
         <v>12</v>
@@ -3336,11 +3464,13 @@
       <c r="F39" s="17"/>
       <c r="G39" s="17"/>
       <c r="H39" s="17" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="I39" s="17"/>
       <c r="J39" s="17"/>
-      <c r="K39" s="17"/>
+      <c r="K39" s="17" t="s">
+        <v>59</v>
+      </c>
       <c r="L39" s="17"/>
       <c r="M39" s="17"/>
       <c r="N39" s="17"/>
@@ -3396,11 +3526,13 @@
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I40" s="2"/>
       <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
+      <c r="K40" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="L40" s="2"/>
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
@@ -3514,11 +3646,13 @@
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="2" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
-      <c r="K42" s="2"/>
+      <c r="K42" s="2" t="s">
+        <v>63</v>
+      </c>
       <c r="L42" s="2"/>
       <c r="M42" s="2"/>
       <c r="N42" s="2"/>
@@ -3625,7 +3759,7 @@
     <row r="44" spans="1:55" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A44" s="26"/>
       <c r="C44" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="2"/>
@@ -3680,7 +3814,7 @@
       <c r="BB44" s="2"/>
       <c r="BC44" s="2"/>
     </row>
-    <row r="45" spans="1:55" s="18" customFormat="1" ht="17.25" thickTop="1" x14ac:dyDescent="0.6">
+    <row r="45" spans="1:55" s="18" customFormat="1" ht="34.15" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A45" s="27"/>
       <c r="C45" s="21" t="s">
         <v>12</v>
@@ -3690,11 +3824,13 @@
       <c r="F45" s="17"/>
       <c r="G45" s="17"/>
       <c r="H45" s="17" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I45" s="17"/>
       <c r="J45" s="17"/>
-      <c r="K45" s="17"/>
+      <c r="K45" s="17" t="s">
+        <v>72</v>
+      </c>
       <c r="L45" s="17"/>
       <c r="M45" s="17"/>
       <c r="N45" s="17"/>
@@ -3750,11 +3886,13 @@
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
       <c r="H46" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
+      <c r="K46" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="L46" s="2"/>
       <c r="M46" s="2"/>
       <c r="N46" s="2"/>
@@ -3868,11 +4006,13 @@
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
       <c r="H48" s="2" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
-      <c r="K48" s="2"/>
+      <c r="K48" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="L48" s="2"/>
       <c r="M48" s="2"/>
       <c r="N48" s="2"/>
@@ -3979,7 +4119,7 @@
     <row r="50" spans="1:55" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A50" s="26"/>
       <c r="C50" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D50" s="3"/>
       <c r="E50" s="2"/>
@@ -4034,7 +4174,7 @@
       <c r="BB50" s="2"/>
       <c r="BC50" s="2"/>
     </row>
-    <row r="51" spans="1:55" s="18" customFormat="1" ht="17.25" thickTop="1" x14ac:dyDescent="0.6">
+    <row r="51" spans="1:55" s="18" customFormat="1" ht="34.15" thickTop="1" x14ac:dyDescent="0.6">
       <c r="A51" s="27"/>
       <c r="C51" s="21" t="s">
         <v>12</v>
@@ -4044,11 +4184,13 @@
       <c r="F51" s="17"/>
       <c r="G51" s="17"/>
       <c r="H51" s="17" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="I51" s="17"/>
       <c r="J51" s="17"/>
-      <c r="K51" s="17"/>
+      <c r="K51" s="17" t="s">
+        <v>73</v>
+      </c>
       <c r="L51" s="17"/>
       <c r="M51" s="17"/>
       <c r="N51" s="17"/>
@@ -4104,11 +4246,13 @@
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
       <c r="H52" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
-      <c r="K52" s="2"/>
+      <c r="K52" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="L52" s="2"/>
       <c r="M52" s="2"/>
       <c r="N52" s="2"/>
@@ -4222,11 +4366,13 @@
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
       <c r="H54" s="2" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
-      <c r="K54" s="2"/>
+      <c r="K54" s="2" t="s">
+        <v>65</v>
+      </c>
       <c r="L54" s="2"/>
       <c r="M54" s="2"/>
       <c r="N54" s="2"/>
@@ -4333,7 +4479,7 @@
     <row r="56" spans="1:55" ht="17.25" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A56" s="26"/>
       <c r="C56" s="11" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="D56" s="3"/>
       <c r="E56" s="2"/>
@@ -4390,10 +4536,10 @@
     </row>
     <row r="57" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A57" s="26"/>
-      <c r="B57" s="38" t="s">
-        <v>24</v>
-      </c>
-      <c r="C57" s="39"/>
+      <c r="B57" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="C57" s="32"/>
       <c r="D57" s="3"/>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
@@ -4449,19 +4595,21 @@
     </row>
     <row r="58" spans="1:55" ht="17.649999999999999" thickTop="1" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A58" s="26"/>
-      <c r="B58" s="42" t="s">
-        <v>25</v>
-      </c>
-      <c r="C58" s="43"/>
+      <c r="B58" s="29" t="s">
+        <v>24</v>
+      </c>
+      <c r="C58" s="30"/>
       <c r="D58" s="3"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="J58" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="K58" s="2"/>
       <c r="L58" s="2"/>
       <c r="M58" s="2"/>
@@ -4511,6 +4659,16 @@
     <row r="59" spans="1:55" ht="17.25" thickTop="1" x14ac:dyDescent="0.6"/>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="D2:M2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="B57:C57"/>
@@ -4521,16 +4679,6 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="D2:M2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A5:C5"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>